<commit_message>
Exclude swaging machine (#84) from inventory — 83 sellable items
The tube swaging machine (R32ELD-380V) is the workshop's own crimping
equipment, not stock for sale, so it is removed from the catalogue,
import file, price list and reconciliation report. Its supplier short-ship
claim (USD 1,700) is noted separately; the on-order claim value now covers
only the 6 short-shipped connectors (USD 246 / LKR 94,600).

All received-stock figures and the 17 reconciliation findings are unchanged
(the machine was on-order at Qty 0 and never counted in stock value).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XGaKdZM6o9DXx3W2ZVdRyr
</commit_message>
<xml_diff>
--- a/Inventory_Import_HS25E1112W1.xlsx
+++ b/Inventory_Import_HS25E1112W1.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J84"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -3099,41 +3099,9 @@
         <v>1774</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="str">
-        <v>R32ELD-380V</v>
-      </c>
-      <c r="B85" t="str">
-        <v>Tube swaging machine</v>
-      </c>
-      <c r="C85" t="str">
-        <v>R32ELD-380V</v>
-      </c>
-      <c r="D85" t="str">
-        <v>1/4"-2"</v>
-      </c>
-      <c r="E85" t="str">
-        <v>Tube swaging machine, crimp 1/4"-2" 6-51mm 4SH, 12 die sets, 4kW, 380V 3ph, 310kg  [ON ORDER — not yet received, shipment HS25E1112W1]</v>
-      </c>
-      <c r="F85">
-        <v>0</v>
-      </c>
-      <c r="G85">
-        <v>0</v>
-      </c>
-      <c r="H85" t="str">
-        <v>Unit</v>
-      </c>
-      <c r="I85">
-        <v>1045296</v>
-      </c>
-      <c r="J85">
-        <v>653310</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J84"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bill 10% below market mid (undercut the market, keep margin)
Set each item's selling price (Inventory.Price — the rate that auto-fills on a
new invoice line) to round(MarketMid × 0.90), floored at landed cost. This bills
a little under the market mid so the customer sees a saving, while margins stay
strong (30% on ferrules, ~75-79% on hose/unions/welds/flanges); no item bills
below cost.

Examples: 4SH 1-1/4" hose 17,100 -> 15,390 · ferrule 00110-04 351 -> 316 ·
union 22611-06-04 720 -> 648 · flange FL-12 1,800 -> 1,620. MarketMid itself is
unchanged, so the invoice comparison now shows Our Price sitting just below the
Market (Mid) column.

- HydraulicHoseRepair.accdb: Price updated on all 83 items
- data/shipment-HS25E1112W1.json + Inventory_Import_HS25E1112W1.xlsx: same rule
  baked into the master + import file

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XGaKdZM6o9DXx3W2ZVdRyr
</commit_message>
<xml_diff>
--- a/Inventory_Import_HS25E1112W1.xlsx
+++ b/Inventory_Import_HS25E1112W1.xlsx
@@ -473,7 +473,7 @@
         <v>m</v>
       </c>
       <c r="I2">
-        <v>770</v>
+        <v>693</v>
       </c>
       <c r="J2">
         <v>144</v>
@@ -508,7 +508,7 @@
         <v>m</v>
       </c>
       <c r="I3">
-        <v>910</v>
+        <v>819</v>
       </c>
       <c r="J3">
         <v>170</v>
@@ -543,7 +543,7 @@
         <v>m</v>
       </c>
       <c r="I4">
-        <v>1050</v>
+        <v>945</v>
       </c>
       <c r="J4">
         <v>196</v>
@@ -578,7 +578,7 @@
         <v>m</v>
       </c>
       <c r="I5">
-        <v>1100</v>
+        <v>990</v>
       </c>
       <c r="J5">
         <v>206</v>
@@ -613,7 +613,7 @@
         <v>m</v>
       </c>
       <c r="I6">
-        <v>1300</v>
+        <v>1170</v>
       </c>
       <c r="J6">
         <v>243</v>
@@ -648,7 +648,7 @@
         <v>m</v>
       </c>
       <c r="I7">
-        <v>1500</v>
+        <v>1350</v>
       </c>
       <c r="J7">
         <v>280</v>
@@ -683,7 +683,7 @@
         <v>m</v>
       </c>
       <c r="I8">
-        <v>1900</v>
+        <v>1710</v>
       </c>
       <c r="J8">
         <v>355</v>
@@ -718,7 +718,7 @@
         <v>m</v>
       </c>
       <c r="I9">
-        <v>2450</v>
+        <v>2205</v>
       </c>
       <c r="J9">
         <v>458</v>
@@ -753,7 +753,7 @@
         <v>m</v>
       </c>
       <c r="I10">
-        <v>3000</v>
+        <v>2700</v>
       </c>
       <c r="J10">
         <v>561</v>
@@ -788,7 +788,7 @@
         <v>m</v>
       </c>
       <c r="I11">
-        <v>4300</v>
+        <v>3870</v>
       </c>
       <c r="J11">
         <v>804</v>
@@ -823,7 +823,7 @@
         <v>m</v>
       </c>
       <c r="I12">
-        <v>6000</v>
+        <v>5400</v>
       </c>
       <c r="J12">
         <v>1122</v>
@@ -858,7 +858,7 @@
         <v>m</v>
       </c>
       <c r="I13">
-        <v>6130</v>
+        <v>5517</v>
       </c>
       <c r="J13">
         <v>1146</v>
@@ -893,7 +893,7 @@
         <v>m</v>
       </c>
       <c r="I14">
-        <v>8550</v>
+        <v>7695</v>
       </c>
       <c r="J14">
         <v>1599</v>
@@ -928,7 +928,7 @@
         <v>m</v>
       </c>
       <c r="I15">
-        <v>12260</v>
+        <v>11034</v>
       </c>
       <c r="J15">
         <v>2292</v>
@@ -963,7 +963,7 @@
         <v>m</v>
       </c>
       <c r="I16">
-        <v>17100</v>
+        <v>15390</v>
       </c>
       <c r="J16">
         <v>3197</v>
@@ -998,7 +998,7 @@
         <v>Nos</v>
       </c>
       <c r="I17">
-        <v>351</v>
+        <v>316</v>
       </c>
       <c r="J17">
         <v>219</v>
@@ -1033,7 +1033,7 @@
         <v>Nos</v>
       </c>
       <c r="I18">
-        <v>389</v>
+        <v>350</v>
       </c>
       <c r="J18">
         <v>243</v>
@@ -1068,7 +1068,7 @@
         <v>Nos</v>
       </c>
       <c r="I19">
-        <v>428</v>
+        <v>385</v>
       </c>
       <c r="J19">
         <v>268</v>
@@ -1103,7 +1103,7 @@
         <v>Nos</v>
       </c>
       <c r="I20">
-        <v>412</v>
+        <v>371</v>
       </c>
       <c r="J20">
         <v>258</v>
@@ -1138,7 +1138,7 @@
         <v>Nos</v>
       </c>
       <c r="I21">
-        <v>458</v>
+        <v>412</v>
       </c>
       <c r="J21">
         <v>286</v>
@@ -1173,7 +1173,7 @@
         <v>Nos</v>
       </c>
       <c r="I22">
-        <v>504</v>
+        <v>454</v>
       </c>
       <c r="J22">
         <v>315</v>
@@ -1208,7 +1208,7 @@
         <v>Nos</v>
       </c>
       <c r="I23">
-        <v>664</v>
+        <v>598</v>
       </c>
       <c r="J23">
         <v>415</v>
@@ -1243,7 +1243,7 @@
         <v>Nos</v>
       </c>
       <c r="I24">
-        <v>1054</v>
+        <v>949</v>
       </c>
       <c r="J24">
         <v>659</v>
@@ -1278,7 +1278,7 @@
         <v>Nos</v>
       </c>
       <c r="I25">
-        <v>1489</v>
+        <v>1340</v>
       </c>
       <c r="J25">
         <v>931</v>
@@ -1313,7 +1313,7 @@
         <v>Nos</v>
       </c>
       <c r="I26">
-        <v>2291</v>
+        <v>2062</v>
       </c>
       <c r="J26">
         <v>1432</v>
@@ -1348,7 +1348,7 @@
         <v>Nos</v>
       </c>
       <c r="I27">
-        <v>3437</v>
+        <v>3093</v>
       </c>
       <c r="J27">
         <v>2148</v>
@@ -1383,7 +1383,7 @@
         <v>Nos</v>
       </c>
       <c r="I28">
-        <v>1581</v>
+        <v>1423</v>
       </c>
       <c r="J28">
         <v>988</v>
@@ -1418,7 +1418,7 @@
         <v>Nos</v>
       </c>
       <c r="I29">
-        <v>2234</v>
+        <v>2011</v>
       </c>
       <c r="J29">
         <v>1396</v>
@@ -1453,7 +1453,7 @@
         <v>Nos</v>
       </c>
       <c r="I30">
-        <v>3437</v>
+        <v>3093</v>
       </c>
       <c r="J30">
         <v>2148</v>
@@ -1488,7 +1488,7 @@
         <v>Nos</v>
       </c>
       <c r="I31">
-        <v>5155</v>
+        <v>4640</v>
       </c>
       <c r="J31">
         <v>3222</v>
@@ -1523,7 +1523,7 @@
         <v>Nos</v>
       </c>
       <c r="I32">
-        <v>620</v>
+        <v>558</v>
       </c>
       <c r="J32">
         <v>138</v>
@@ -1558,7 +1558,7 @@
         <v>Nos</v>
       </c>
       <c r="I33">
-        <v>720</v>
+        <v>648</v>
       </c>
       <c r="J33">
         <v>161</v>
@@ -1593,7 +1593,7 @@
         <v>Nos</v>
       </c>
       <c r="I34">
-        <v>720</v>
+        <v>648</v>
       </c>
       <c r="J34">
         <v>161</v>
@@ -1628,7 +1628,7 @@
         <v>Nos</v>
       </c>
       <c r="I35">
-        <v>720</v>
+        <v>648</v>
       </c>
       <c r="J35">
         <v>161</v>
@@ -1663,7 +1663,7 @@
         <v>Nos</v>
       </c>
       <c r="I36">
-        <v>950</v>
+        <v>855</v>
       </c>
       <c r="J36">
         <v>212</v>
@@ -1698,7 +1698,7 @@
         <v>Nos</v>
       </c>
       <c r="I37">
-        <v>950</v>
+        <v>855</v>
       </c>
       <c r="J37">
         <v>212</v>
@@ -1733,7 +1733,7 @@
         <v>Nos</v>
       </c>
       <c r="I38">
-        <v>1250</v>
+        <v>1125</v>
       </c>
       <c r="J38">
         <v>279</v>
@@ -1768,7 +1768,7 @@
         <v>Nos</v>
       </c>
       <c r="I39">
-        <v>1600</v>
+        <v>1440</v>
       </c>
       <c r="J39">
         <v>357</v>
@@ -1803,7 +1803,7 @@
         <v>Nos</v>
       </c>
       <c r="I40">
-        <v>2600</v>
+        <v>2340</v>
       </c>
       <c r="J40">
         <v>581</v>
@@ -1838,7 +1838,7 @@
         <v>Nos</v>
       </c>
       <c r="I41">
-        <v>3900</v>
+        <v>3510</v>
       </c>
       <c r="J41">
         <v>871</v>
@@ -1873,7 +1873,7 @@
         <v>Nos</v>
       </c>
       <c r="I42">
-        <v>1209</v>
+        <v>1088</v>
       </c>
       <c r="J42">
         <v>270</v>
@@ -1908,7 +1908,7 @@
         <v>Nos</v>
       </c>
       <c r="I43">
-        <v>1404</v>
+        <v>1264</v>
       </c>
       <c r="J43">
         <v>314</v>
@@ -1943,7 +1943,7 @@
         <v>Nos</v>
       </c>
       <c r="I44">
-        <v>1852</v>
+        <v>1667</v>
       </c>
       <c r="J44">
         <v>414</v>
@@ -1978,7 +1978,7 @@
         <v>Nos</v>
       </c>
       <c r="I45">
-        <v>713</v>
+        <v>642</v>
       </c>
       <c r="J45">
         <v>159</v>
@@ -2013,7 +2013,7 @@
         <v>Nos</v>
       </c>
       <c r="I46">
-        <v>828</v>
+        <v>745</v>
       </c>
       <c r="J46">
         <v>185</v>
@@ -2048,7 +2048,7 @@
         <v>Nos</v>
       </c>
       <c r="I47">
-        <v>1092</v>
+        <v>983</v>
       </c>
       <c r="J47">
         <v>244</v>
@@ -2083,7 +2083,7 @@
         <v>Nos</v>
       </c>
       <c r="I48">
-        <v>1840</v>
+        <v>1656</v>
       </c>
       <c r="J48">
         <v>411</v>
@@ -2118,7 +2118,7 @@
         <v>Nos</v>
       </c>
       <c r="I49">
-        <v>2990</v>
+        <v>2691</v>
       </c>
       <c r="J49">
         <v>668</v>
@@ -2153,7 +2153,7 @@
         <v>Nos</v>
       </c>
       <c r="I50">
-        <v>4485</v>
+        <v>4037</v>
       </c>
       <c r="J50">
         <v>1002</v>
@@ -2188,7 +2188,7 @@
         <v>Nos</v>
       </c>
       <c r="I51">
-        <v>1250</v>
+        <v>1125</v>
       </c>
       <c r="J51">
         <v>315</v>
@@ -2223,7 +2223,7 @@
         <v>Nos</v>
       </c>
       <c r="I52">
-        <v>1600</v>
+        <v>1440</v>
       </c>
       <c r="J52">
         <v>404</v>
@@ -2258,7 +2258,7 @@
         <v>Nos</v>
       </c>
       <c r="I53">
-        <v>2600</v>
+        <v>2340</v>
       </c>
       <c r="J53">
         <v>656</v>
@@ -2293,7 +2293,7 @@
         <v>Nos</v>
       </c>
       <c r="I54">
-        <v>3900</v>
+        <v>3510</v>
       </c>
       <c r="J54">
         <v>984</v>
@@ -2328,7 +2328,7 @@
         <v>Nos</v>
       </c>
       <c r="I55">
-        <v>1209</v>
+        <v>1088</v>
       </c>
       <c r="J55">
         <v>305</v>
@@ -2363,7 +2363,7 @@
         <v>Nos</v>
       </c>
       <c r="I56">
-        <v>1404</v>
+        <v>1264</v>
       </c>
       <c r="J56">
         <v>354</v>
@@ -2398,7 +2398,7 @@
         <v>Nos</v>
       </c>
       <c r="I57">
-        <v>1852</v>
+        <v>1667</v>
       </c>
       <c r="J57">
         <v>467</v>
@@ -2433,7 +2433,7 @@
         <v>Nos</v>
       </c>
       <c r="I58">
-        <v>2438</v>
+        <v>2194</v>
       </c>
       <c r="J58">
         <v>615</v>
@@ -2468,7 +2468,7 @@
         <v>Nos</v>
       </c>
       <c r="I59">
-        <v>3120</v>
+        <v>2808</v>
       </c>
       <c r="J59">
         <v>787</v>
@@ -2503,7 +2503,7 @@
         <v>Nos</v>
       </c>
       <c r="I60">
-        <v>5070</v>
+        <v>4563</v>
       </c>
       <c r="J60">
         <v>1279</v>
@@ -2538,7 +2538,7 @@
         <v>Nos</v>
       </c>
       <c r="I61">
-        <v>7605</v>
+        <v>6845</v>
       </c>
       <c r="J61">
         <v>1918</v>
@@ -2573,7 +2573,7 @@
         <v>Nos</v>
       </c>
       <c r="I62">
-        <v>372</v>
+        <v>335</v>
       </c>
       <c r="J62">
         <v>70</v>
@@ -2608,7 +2608,7 @@
         <v>Nos</v>
       </c>
       <c r="I63">
-        <v>402</v>
+        <v>362</v>
       </c>
       <c r="J63">
         <v>76</v>
@@ -2643,7 +2643,7 @@
         <v>Nos</v>
       </c>
       <c r="I64">
-        <v>432</v>
+        <v>389</v>
       </c>
       <c r="J64">
         <v>82</v>
@@ -2678,7 +2678,7 @@
         <v>Nos</v>
       </c>
       <c r="I65">
-        <v>570</v>
+        <v>513</v>
       </c>
       <c r="J65">
         <v>108</v>
@@ -2713,7 +2713,7 @@
         <v>Nos</v>
       </c>
       <c r="I66">
-        <v>750</v>
+        <v>675</v>
       </c>
       <c r="J66">
         <v>142</v>
@@ -2748,7 +2748,7 @@
         <v>Nos</v>
       </c>
       <c r="I67">
-        <v>960</v>
+        <v>864</v>
       </c>
       <c r="J67">
         <v>182</v>
@@ -2783,7 +2783,7 @@
         <v>Nos</v>
       </c>
       <c r="I68">
-        <v>1560</v>
+        <v>1404</v>
       </c>
       <c r="J68">
         <v>295</v>
@@ -2818,7 +2818,7 @@
         <v>Nos</v>
       </c>
       <c r="I69">
-        <v>2340</v>
+        <v>2106</v>
       </c>
       <c r="J69">
         <v>443</v>
@@ -2853,7 +2853,7 @@
         <v>Nos</v>
       </c>
       <c r="I70">
-        <v>558</v>
+        <v>502</v>
       </c>
       <c r="J70">
         <v>171</v>
@@ -2888,7 +2888,7 @@
         <v>Nos</v>
       </c>
       <c r="I71">
-        <v>648</v>
+        <v>583</v>
       </c>
       <c r="J71">
         <v>198</v>
@@ -2923,7 +2923,7 @@
         <v>Nos</v>
       </c>
       <c r="I72">
-        <v>855</v>
+        <v>770</v>
       </c>
       <c r="J72">
         <v>262</v>
@@ -2958,7 +2958,7 @@
         <v>Nos</v>
       </c>
       <c r="I73">
-        <v>1125</v>
+        <v>1013</v>
       </c>
       <c r="J73">
         <v>344</v>
@@ -2993,7 +2993,7 @@
         <v>Nos</v>
       </c>
       <c r="I74">
-        <v>806</v>
+        <v>725</v>
       </c>
       <c r="J74">
         <v>289</v>
@@ -3028,7 +3028,7 @@
         <v>Nos</v>
       </c>
       <c r="I75">
-        <v>806</v>
+        <v>725</v>
       </c>
       <c r="J75">
         <v>289</v>
@@ -3063,7 +3063,7 @@
         <v>Nos</v>
       </c>
       <c r="I76">
-        <v>936</v>
+        <v>842</v>
       </c>
       <c r="J76">
         <v>335</v>
@@ -3098,7 +3098,7 @@
         <v>Nos</v>
       </c>
       <c r="I77">
-        <v>1235</v>
+        <v>1112</v>
       </c>
       <c r="J77">
         <v>442</v>
@@ -3133,7 +3133,7 @@
         <v>Nos</v>
       </c>
       <c r="I78">
-        <v>950</v>
+        <v>855</v>
       </c>
       <c r="J78">
         <v>362</v>
@@ -3168,7 +3168,7 @@
         <v>Nos</v>
       </c>
       <c r="I79">
-        <v>950</v>
+        <v>855</v>
       </c>
       <c r="J79">
         <v>362</v>
@@ -3203,7 +3203,7 @@
         <v>Nos</v>
       </c>
       <c r="I80">
-        <v>1800</v>
+        <v>1620</v>
       </c>
       <c r="J80">
         <v>394</v>
@@ -3238,7 +3238,7 @@
         <v>Nos</v>
       </c>
       <c r="I81">
-        <v>2520</v>
+        <v>2268</v>
       </c>
       <c r="J81">
         <v>552</v>
@@ -3273,7 +3273,7 @@
         <v>Nos</v>
       </c>
       <c r="I82">
-        <v>3240</v>
+        <v>2916</v>
       </c>
       <c r="J82">
         <v>709</v>
@@ -3308,7 +3308,7 @@
         <v>Nos</v>
       </c>
       <c r="I83">
-        <v>4350</v>
+        <v>3915</v>
       </c>
       <c r="J83">
         <v>1182</v>
@@ -3343,7 +3343,7 @@
         <v>Nos</v>
       </c>
       <c r="I84">
-        <v>6525</v>
+        <v>5873</v>
       </c>
       <c r="J84">
         <v>1774</v>

</xml_diff>